<commit_message>
refactor: simplify test data usage and remove unnecessary logs
</commit_message>
<xml_diff>
--- a/src/test/resources/massa/Massa/automationExercise.xlsx
+++ b/src/test/resources/massa/Massa/automationExercise.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="17">
   <si>
     <t>CT</t>
   </si>
@@ -31,6 +31,9 @@
     <t>MESSAGE</t>
   </si>
   <si>
+    <t>PRODUCT</t>
+  </si>
+  <si>
     <t>1</t>
   </si>
   <si>
@@ -47,6 +50,9 @@
   </si>
   <si>
     <t>2</t>
+  </si>
+  <si>
+    <t>Polo</t>
   </si>
   <si>
     <t>sdadsadsdad@a.com</t>
@@ -379,7 +385,9 @@
       <c r="F1" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="3"/>
+      <c r="G1" s="2" t="s">
+        <v>6</v>
+      </c>
       <c r="H1" s="3"/>
       <c r="I1" s="3"/>
       <c r="J1" s="3"/>
@@ -402,22 +410,22 @@
     </row>
     <row r="2">
       <c r="A2" s="4" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F2" s="5" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="G2" s="3"/>
       <c r="H2" s="3"/>
@@ -442,18 +450,20 @@
     </row>
     <row r="3">
       <c r="A3" s="4" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D3" s="6"/>
       <c r="E3" s="3"/>
       <c r="F3" s="3"/>
-      <c r="G3" s="3"/>
+      <c r="G3" s="2" t="s">
+        <v>13</v>
+      </c>
       <c r="H3" s="3"/>
       <c r="I3" s="3"/>
       <c r="J3" s="3"/>
@@ -479,10 +489,10 @@
         <v>3.0</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="D4" s="6"/>
       <c r="E4" s="3"/>
@@ -510,14 +520,14 @@
     </row>
     <row r="5">
       <c r="A5" s="4" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C5" s="6"/>
       <c r="D5" s="1" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="E5" s="3"/>
       <c r="F5" s="3"/>

</xml_diff>

<commit_message>
feat: add cart validation after login
</commit_message>
<xml_diff>
--- a/src/test/resources/massa/Massa/automationExercise.xlsx
+++ b/src/test/resources/massa/Massa/automationExercise.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="22">
   <si>
     <t>CT</t>
   </si>
@@ -132,7 +132,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -147,6 +147,9 @@
     </xf>
     <xf borderId="1" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center"/>
@@ -552,9 +555,15 @@
       </c>
       <c r="E5" s="4"/>
       <c r="F5" s="4"/>
-      <c r="G5" s="4"/>
-      <c r="H5" s="4"/>
-      <c r="I5" s="4"/>
+      <c r="G5" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="H5" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="I5" s="1" t="s">
+        <v>20</v>
+      </c>
       <c r="J5" s="2"/>
       <c r="K5" s="2"/>
       <c r="L5" s="2"/>
@@ -574,10 +583,16 @@
       <c r="Z5" s="2"/>
     </row>
     <row r="6">
-      <c r="A6" s="5"/>
-      <c r="B6" s="2"/>
-      <c r="C6" s="2"/>
-      <c r="D6" s="2"/>
+      <c r="A6" s="5">
+        <v>5.0</v>
+      </c>
+      <c r="B6" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D6" s="5"/>
       <c r="E6" s="2"/>
       <c r="F6" s="2"/>
       <c r="G6" s="2"/>
@@ -602,11 +617,11 @@
       <c r="Z6" s="2"/>
     </row>
     <row r="7">
-      <c r="A7" s="2"/>
+      <c r="A7" s="6"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
       <c r="D7" s="2"/>
-      <c r="E7" s="5"/>
+      <c r="E7" s="2"/>
       <c r="F7" s="2"/>
       <c r="G7" s="2"/>
       <c r="H7" s="2"/>
@@ -634,7 +649,7 @@
       <c r="B8" s="2"/>
       <c r="C8" s="2"/>
       <c r="D8" s="2"/>
-      <c r="E8" s="2"/>
+      <c r="E8" s="6"/>
       <c r="F8" s="2"/>
       <c r="G8" s="2"/>
       <c r="H8" s="2"/>
@@ -746,7 +761,7 @@
       <c r="B12" s="2"/>
       <c r="C12" s="2"/>
       <c r="D12" s="2"/>
-      <c r="E12" s="5"/>
+      <c r="E12" s="2"/>
       <c r="F12" s="2"/>
       <c r="G12" s="2"/>
       <c r="H12" s="2"/>
@@ -773,8 +788,8 @@
       <c r="A13" s="2"/>
       <c r="B13" s="2"/>
       <c r="C13" s="2"/>
-      <c r="D13" s="5"/>
-      <c r="E13" s="2"/>
+      <c r="D13" s="2"/>
+      <c r="E13" s="6"/>
       <c r="F13" s="2"/>
       <c r="G13" s="2"/>
       <c r="H13" s="2"/>
@@ -801,7 +816,7 @@
       <c r="A14" s="2"/>
       <c r="B14" s="2"/>
       <c r="C14" s="2"/>
-      <c r="D14" s="2"/>
+      <c r="D14" s="6"/>
       <c r="E14" s="2"/>
       <c r="F14" s="2"/>
       <c r="G14" s="2"/>
@@ -1558,7 +1573,7 @@
       <c r="B41" s="2"/>
       <c r="C41" s="2"/>
       <c r="D41" s="2"/>
-      <c r="E41" s="5"/>
+      <c r="E41" s="2"/>
       <c r="F41" s="2"/>
       <c r="G41" s="2"/>
       <c r="H41" s="2"/>
@@ -1586,7 +1601,7 @@
       <c r="B42" s="2"/>
       <c r="C42" s="2"/>
       <c r="D42" s="2"/>
-      <c r="E42" s="2"/>
+      <c r="E42" s="6"/>
       <c r="F42" s="2"/>
       <c r="G42" s="2"/>
       <c r="H42" s="2"/>
@@ -28433,6 +28448,34 @@
       <c r="Y1000" s="2"/>
       <c r="Z1000" s="2"/>
     </row>
+    <row r="1001">
+      <c r="A1001" s="2"/>
+      <c r="B1001" s="2"/>
+      <c r="C1001" s="2"/>
+      <c r="D1001" s="2"/>
+      <c r="E1001" s="2"/>
+      <c r="F1001" s="2"/>
+      <c r="G1001" s="2"/>
+      <c r="H1001" s="2"/>
+      <c r="I1001" s="2"/>
+      <c r="J1001" s="2"/>
+      <c r="K1001" s="2"/>
+      <c r="L1001" s="2"/>
+      <c r="M1001" s="2"/>
+      <c r="N1001" s="2"/>
+      <c r="O1001" s="2"/>
+      <c r="P1001" s="2"/>
+      <c r="Q1001" s="2"/>
+      <c r="R1001" s="2"/>
+      <c r="S1001" s="2"/>
+      <c r="T1001" s="2"/>
+      <c r="U1001" s="2"/>
+      <c r="V1001" s="2"/>
+      <c r="W1001" s="2"/>
+      <c r="X1001" s="2"/>
+      <c r="Y1001" s="2"/>
+      <c r="Z1001" s="2"/>
+    </row>
   </sheetData>
   <drawing r:id="rId1"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: add remove product from cart scenario
</commit_message>
<xml_diff>
--- a/src/test/resources/massa/Massa/automationExercise.xlsx
+++ b/src/test/resources/massa/Massa/automationExercise.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="22">
   <si>
     <t>CT</t>
   </si>
@@ -595,9 +595,15 @@
       <c r="D6" s="5"/>
       <c r="E6" s="2"/>
       <c r="F6" s="2"/>
-      <c r="G6" s="2"/>
-      <c r="H6" s="2"/>
-      <c r="I6" s="2"/>
+      <c r="G6" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="H6" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="I6" s="1" t="s">
+        <v>20</v>
+      </c>
       <c r="J6" s="2"/>
       <c r="K6" s="2"/>
       <c r="L6" s="2"/>

</xml_diff>

<commit_message>
feat: add product review scenario
</commit_message>
<xml_diff>
--- a/src/test/resources/massa/Massa/automationExercise.xlsx
+++ b/src/test/resources/massa/Massa/automationExercise.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="23">
   <si>
     <t>CT</t>
   </si>
@@ -77,6 +77,9 @@
   </si>
   <si>
     <t>4</t>
+  </si>
+  <si>
+    <t>TESTE</t>
   </si>
 </sst>
 </file>
@@ -148,7 +151,7 @@
     <xf borderId="1" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="1" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
@@ -583,18 +586,18 @@
       <c r="Z5" s="2"/>
     </row>
     <row r="6">
-      <c r="A6" s="5">
+      <c r="A6" s="1">
         <v>5.0</v>
       </c>
-      <c r="B6" s="5" t="s">
+      <c r="B6" s="1" t="s">
         <v>10</v>
       </c>
       <c r="C6" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="D6" s="5"/>
-      <c r="E6" s="2"/>
-      <c r="F6" s="2"/>
+      <c r="D6" s="1"/>
+      <c r="E6" s="4"/>
+      <c r="F6" s="4"/>
       <c r="G6" s="1" t="s">
         <v>18</v>
       </c>
@@ -623,15 +626,23 @@
       <c r="Z6" s="2"/>
     </row>
     <row r="7">
-      <c r="A7" s="6"/>
-      <c r="B7" s="2"/>
-      <c r="C7" s="2"/>
-      <c r="D7" s="2"/>
-      <c r="E7" s="2"/>
-      <c r="F7" s="2"/>
-      <c r="G7" s="2"/>
-      <c r="H7" s="2"/>
-      <c r="I7" s="2"/>
+      <c r="A7" s="5">
+        <v>6.0</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C7" s="4"/>
+      <c r="D7" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="E7" s="4"/>
+      <c r="F7" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="G7" s="4"/>
+      <c r="H7" s="4"/>
+      <c r="I7" s="4"/>
       <c r="J7" s="2"/>
       <c r="K7" s="2"/>
       <c r="L7" s="2"/>
@@ -652,11 +663,8 @@
     </row>
     <row r="8">
       <c r="A8" s="2"/>
-      <c r="B8" s="2"/>
       <c r="C8" s="2"/>
-      <c r="D8" s="2"/>
       <c r="E8" s="6"/>
-      <c r="F8" s="2"/>
       <c r="G8" s="2"/>
       <c r="H8" s="2"/>
       <c r="I8" s="2"/>

</xml_diff>

<commit_message>
fix: wait for product removal before cart validation
</commit_message>
<xml_diff>
--- a/src/test/resources/massa/Massa/automationExercise.xlsx
+++ b/src/test/resources/massa/Massa/automationExercise.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="23">
   <si>
     <t>CT</t>
   </si>
@@ -86,7 +86,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <fonts count="3">
+  <fonts count="4">
     <font>
       <sz val="10.0"/>
       <color rgb="FF000000"/>
@@ -102,6 +102,11 @@
     <font>
       <b/>
       <sz val="18.0"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <color theme="1"/>
       <name val="Arial"/>
       <scheme val="minor"/>
@@ -135,7 +140,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="9">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -154,6 +159,10 @@
     <xf borderId="1" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
+    <xf borderId="1" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf borderId="1" fillId="0" fontId="3" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center"/>
     </xf>
@@ -378,7 +387,8 @@
     <col customWidth="1" min="2" max="2" width="35.88"/>
     <col customWidth="1" min="3" max="5" width="31.13"/>
     <col customWidth="1" min="6" max="6" width="30.0"/>
-    <col customWidth="1" min="7" max="8" width="31.13"/>
+    <col customWidth="1" min="7" max="7" width="31.0"/>
+    <col customWidth="1" min="8" max="8" width="31.13"/>
     <col customWidth="1" min="9" max="9" width="37.13"/>
     <col customWidth="1" min="10" max="26" width="31.13"/>
   </cols>
@@ -662,12 +672,29 @@
       <c r="Z7" s="2"/>
     </row>
     <row r="8">
-      <c r="A8" s="2"/>
-      <c r="C8" s="2"/>
+      <c r="A8" s="1">
+        <v>7.0</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>22</v>
+      </c>
       <c r="E8" s="6"/>
-      <c r="G8" s="2"/>
-      <c r="H8" s="2"/>
-      <c r="I8" s="2"/>
+      <c r="F8" s="7"/>
+      <c r="G8" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="H8" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="I8" s="1" t="s">
+        <v>20</v>
+      </c>
       <c r="J8" s="2"/>
       <c r="K8" s="2"/>
       <c r="L8" s="2"/>
@@ -803,7 +830,7 @@
       <c r="B13" s="2"/>
       <c r="C13" s="2"/>
       <c r="D13" s="2"/>
-      <c r="E13" s="6"/>
+      <c r="E13" s="8"/>
       <c r="F13" s="2"/>
       <c r="G13" s="2"/>
       <c r="H13" s="2"/>
@@ -830,7 +857,7 @@
       <c r="A14" s="2"/>
       <c r="B14" s="2"/>
       <c r="C14" s="2"/>
-      <c r="D14" s="6"/>
+      <c r="D14" s="8"/>
       <c r="E14" s="2"/>
       <c r="F14" s="2"/>
       <c r="G14" s="2"/>
@@ -1615,7 +1642,7 @@
       <c r="B42" s="2"/>
       <c r="C42" s="2"/>
       <c r="D42" s="2"/>
-      <c r="E42" s="6"/>
+      <c r="E42" s="8"/>
       <c r="F42" s="2"/>
       <c r="G42" s="2"/>
       <c r="H42" s="2"/>

</xml_diff>